<commit_message>
Refactor version handling in Frame and Signal services
- Removed deprecated version comparison logic and replaced it with nextVersionId checks for filtering active versions.
- Updated Frame and Signal interfaces to include previousVersionId and nextVersionId fields.
- Modified various services (ApplicationService, CommunicationDataReflectionService, EcuPortMatrixService, etc.) to utilize new versioning logic.
- Enhanced frame and signal resolution functions to ensure only the latest non-deleted versions are processed.
- Implemented carry-over logic for signals when frames are updated without changes.
- Cleaned up unused imports and functions related to version comparison.
</commit_message>
<xml_diff>
--- a/samples/通信データExcel_サンプル - コピー.xlsx
+++ b/samples/通信データExcel_サンプル - コピー.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="64">
   <si>
     <t xml:space="preserve">Engine_10_CONN_E2</t>
   </si>
@@ -490,24 +490,6 @@
   </si>
   <si>
     <t xml:space="preserve">km/h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frame_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">エンジン</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00-b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signal_EngineSpeed2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01-a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Signal_VehicleSpeed2</t>
   </si>
 </sst>
 </file>
@@ -802,7 +784,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AS8"/>
+  <dimension ref="A1:AS10"/>
   <sheetFormatPr defaultColWidth="7.796875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1184,237 +1166,17 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" s="0" t="n">
-        <v>32</v>
-      </c>
-      <c r="L6" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="T6" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AH6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AL6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AM6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AN6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AO6" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="AP6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AQ6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AR6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AS6" s="0" t="n">
-        <v>200</v>
-      </c>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="29.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="Y7" s="0" t="n">
-        <v>24</v>
-      </c>
-      <c r="Z7" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB7" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AC7" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD7" s="0" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="AE7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" s="0" t="n">
-        <v>65535</v>
-      </c>
-      <c r="AG7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AH7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AL7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AM7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AN7" s="1" t="s">
-        <v>54</v>
-      </c>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="29.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y8" s="0" t="n">
-        <v>40</v>
-      </c>
-      <c r="Z8" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AC8" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="AD8" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AE8" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" s="0" t="n">
-        <v>65535</v>
-      </c>
-      <c r="AG8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AH8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AJ8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AL8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AM8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AN8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AP8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AQ8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AR8" s="1" t="s">
-        <v>54</v>
-      </c>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="2"/>
     </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>